<commit_message>
fix: corrige nome do autor — Ilson do Santos Azevedo / Supervisor de Planejamento
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168LAty28evK8EwJcgZFrtt
</commit_message>
<xml_diff>
--- a/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
+++ b/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
@@ -579,7 +579,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV1 — 03/07/2026  |  Elaborado por: Ilson dos Santos Azevedo — Supervisor de Planejamento</t>
+          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV1 — 03/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
         </is>
       </c>
     </row>
@@ -7869,12 +7869,12 @@
     <mergeCell ref="B63:B66"/>
     <mergeCell ref="E23:E31"/>
     <mergeCell ref="D111:D117"/>
+    <mergeCell ref="E143:E149"/>
     <mergeCell ref="D63:D66"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="D10:D13"/>
+    <mergeCell ref="C189:C194"/>
     <mergeCell ref="C143:C149"/>
-    <mergeCell ref="E143:E149"/>
-    <mergeCell ref="C189:C194"/>
     <mergeCell ref="E189:E194"/>
     <mergeCell ref="B14:B22"/>
     <mergeCell ref="A36:A39"/>
@@ -7926,7 +7926,6 @@
     <mergeCell ref="E180:E182"/>
     <mergeCell ref="B93:B99"/>
     <mergeCell ref="M63:M66"/>
-    <mergeCell ref="C205:C206"/>
     <mergeCell ref="B32:B35"/>
     <mergeCell ref="A207:A208"/>
     <mergeCell ref="A67:A70"/>
@@ -7992,6 +7991,7 @@
     <mergeCell ref="A209:A211"/>
     <mergeCell ref="C209:C211"/>
     <mergeCell ref="B82:B92"/>
+    <mergeCell ref="C205:C206"/>
     <mergeCell ref="D143:D149"/>
     <mergeCell ref="C63:C66"/>
     <mergeCell ref="M67:M70"/>

</xml_diff>

<commit_message>
feat: PUSH LIST REV2 — foto largura total, KPIs simplificados, Platô Central
- Foto largura total no card (260px altura, card inteiro)
- Mini velocímetro por card mantido abaixo da foto (menos intrusivo)
- Velocímetro único global no KPI mostrando Avanço Físico
- Remove KPIs: Total Peso, Avanço Ponderado, Área Mais Crítica, Disciplina em Atraso
- Gráfico de disciplinas melhorado (SVG colorido com barras proporcionais)
- Platô Central: 3 fotos incluídas (03/07/2026) — 38 cards no total
- Placeholder Curva-S (ativa quando Lucas lançar datas)
- Footer: Ilson do Santos Azevedo / Supervisor de Planejamento

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168LAty28evK8EwJcgZFrtt
</commit_message>
<xml_diff>
--- a/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
+++ b/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Push List REV1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Push List REV2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M211"/>
+  <dimension ref="A1:M217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -579,7 +579,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV1 — 03/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
+          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV2 — 03/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
         </is>
       </c>
     </row>
@@ -7724,10 +7724,8 @@
           <t>Platô Central</t>
         </is>
       </c>
-      <c r="E209" s="9" t="inlineStr">
-        <is>
-          <t>S/F</t>
-        </is>
+      <c r="E209" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="F209" s="9" t="n">
         <v>1</v>
@@ -7820,8 +7818,234 @@
       <c r="L211" s="9" t="inlineStr"/>
       <c r="M211" s="12" t="n"/>
     </row>
+    <row r="212" ht="16" customHeight="1">
+      <c r="A212" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B212" s="5" t="inlineStr">
+        <is>
+          <t>Platô Central</t>
+        </is>
+      </c>
+      <c r="C212" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D212" s="5" t="inlineStr">
+        <is>
+          <t>Platô Central</t>
+        </is>
+      </c>
+      <c r="E212" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F212" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G212" s="6" t="inlineStr">
+        <is>
+          <t>Macrodrenagem</t>
+        </is>
+      </c>
+      <c r="H212" s="7" t="inlineStr">
+        <is>
+          <t>Remoção de Canaletas</t>
+        </is>
+      </c>
+      <c r="I212" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J212" s="4" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K212" s="4" t="inlineStr"/>
+      <c r="L212" s="4" t="inlineStr"/>
+      <c r="M212" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="16" customHeight="1">
+      <c r="A213" s="8" t="n"/>
+      <c r="B213" s="8" t="n"/>
+      <c r="C213" s="8" t="n"/>
+      <c r="D213" s="8" t="n"/>
+      <c r="E213" s="8" t="n"/>
+      <c r="F213" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G213" s="10" t="inlineStr">
+        <is>
+          <t>Terraplanagem</t>
+        </is>
+      </c>
+      <c r="H213" s="11" t="inlineStr">
+        <is>
+          <t>Regularização e adensamento do Platôr Central</t>
+        </is>
+      </c>
+      <c r="I213" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J213" s="9" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K213" s="9" t="inlineStr"/>
+      <c r="L213" s="9" t="inlineStr"/>
+      <c r="M213" s="8" t="n"/>
+    </row>
+    <row r="214" ht="16" customHeight="1">
+      <c r="A214" s="12" t="n"/>
+      <c r="B214" s="12" t="n"/>
+      <c r="C214" s="12" t="n"/>
+      <c r="D214" s="12" t="n"/>
+      <c r="E214" s="12" t="n"/>
+      <c r="F214" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G214" s="6" t="inlineStr">
+        <is>
+          <t>Geral / 5S</t>
+        </is>
+      </c>
+      <c r="H214" s="7" t="inlineStr">
+        <is>
+          <t>Limpeza geral e reorganização da área</t>
+        </is>
+      </c>
+      <c r="I214" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J214" s="4" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K214" s="4" t="inlineStr"/>
+      <c r="L214" s="4" t="inlineStr"/>
+      <c r="M214" s="12" t="n"/>
+    </row>
+    <row r="215" ht="16" customHeight="1">
+      <c r="A215" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="B215" s="13" t="inlineStr">
+        <is>
+          <t>Platô Central</t>
+        </is>
+      </c>
+      <c r="C215" s="9" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D215" s="13" t="inlineStr">
+        <is>
+          <t>Platô Central</t>
+        </is>
+      </c>
+      <c r="E215" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F215" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G215" s="10" t="inlineStr">
+        <is>
+          <t>Macrodrenagem</t>
+        </is>
+      </c>
+      <c r="H215" s="11" t="inlineStr">
+        <is>
+          <t>Remoção de Canaletas</t>
+        </is>
+      </c>
+      <c r="I215" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J215" s="9" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K215" s="9" t="inlineStr"/>
+      <c r="L215" s="9" t="inlineStr"/>
+      <c r="M215" s="9" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="16" customHeight="1">
+      <c r="A216" s="8" t="n"/>
+      <c r="B216" s="8" t="n"/>
+      <c r="C216" s="8" t="n"/>
+      <c r="D216" s="8" t="n"/>
+      <c r="E216" s="8" t="n"/>
+      <c r="F216" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G216" s="6" t="inlineStr">
+        <is>
+          <t>Terraplanagem</t>
+        </is>
+      </c>
+      <c r="H216" s="7" t="inlineStr">
+        <is>
+          <t>Regularização e adensamento do Platôr Central</t>
+        </is>
+      </c>
+      <c r="I216" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J216" s="4" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K216" s="4" t="inlineStr"/>
+      <c r="L216" s="4" t="inlineStr"/>
+      <c r="M216" s="8" t="n"/>
+    </row>
+    <row r="217" ht="16" customHeight="1">
+      <c r="A217" s="12" t="n"/>
+      <c r="B217" s="12" t="n"/>
+      <c r="C217" s="12" t="n"/>
+      <c r="D217" s="12" t="n"/>
+      <c r="E217" s="12" t="n"/>
+      <c r="F217" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G217" s="10" t="inlineStr">
+        <is>
+          <t>Geral / 5S</t>
+        </is>
+      </c>
+      <c r="H217" s="11" t="inlineStr">
+        <is>
+          <t>Limpeza geral e reorganização da área</t>
+        </is>
+      </c>
+      <c r="I217" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J217" s="9" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K217" s="9" t="inlineStr"/>
+      <c r="L217" s="9" t="inlineStr"/>
+      <c r="M217" s="12" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="218">
+  <mergeCells count="230">
     <mergeCell ref="E203:E204"/>
     <mergeCell ref="B50:B55"/>
     <mergeCell ref="E118:E124"/>
@@ -7829,6 +8053,7 @@
     <mergeCell ref="D180:D182"/>
     <mergeCell ref="E183:E188"/>
     <mergeCell ref="A136:A142"/>
+    <mergeCell ref="D212:D214"/>
     <mergeCell ref="M50:M55"/>
     <mergeCell ref="D46:D49"/>
     <mergeCell ref="M203:M204"/>
@@ -7846,6 +8071,7 @@
     <mergeCell ref="M14:M22"/>
     <mergeCell ref="A125:A135"/>
     <mergeCell ref="E207:E208"/>
+    <mergeCell ref="B215:B217"/>
     <mergeCell ref="M36:M39"/>
     <mergeCell ref="B205:B206"/>
     <mergeCell ref="A203:A204"/>
@@ -7853,10 +8079,14 @@
     <mergeCell ref="D157:D167"/>
     <mergeCell ref="E125:E135"/>
     <mergeCell ref="A195:A200"/>
+    <mergeCell ref="A212:A214"/>
     <mergeCell ref="D168:D173"/>
+    <mergeCell ref="C212:C214"/>
     <mergeCell ref="A63:A66"/>
     <mergeCell ref="E100:E110"/>
     <mergeCell ref="A10:A13"/>
+    <mergeCell ref="C215:C217"/>
+    <mergeCell ref="E215:E217"/>
     <mergeCell ref="M71:M81"/>
     <mergeCell ref="A174:A176"/>
     <mergeCell ref="B100:B110"/>
@@ -7869,12 +8099,12 @@
     <mergeCell ref="B63:B66"/>
     <mergeCell ref="E23:E31"/>
     <mergeCell ref="D111:D117"/>
-    <mergeCell ref="E143:E149"/>
     <mergeCell ref="D63:D66"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="D10:D13"/>
+    <mergeCell ref="C143:C149"/>
+    <mergeCell ref="E143:E149"/>
     <mergeCell ref="C189:C194"/>
-    <mergeCell ref="C143:C149"/>
     <mergeCell ref="E189:E194"/>
     <mergeCell ref="B14:B22"/>
     <mergeCell ref="A36:A39"/>
@@ -7924,8 +8154,10 @@
     <mergeCell ref="C180:C182"/>
     <mergeCell ref="A4:A9"/>
     <mergeCell ref="E180:E182"/>
+    <mergeCell ref="M212:M214"/>
     <mergeCell ref="B93:B99"/>
     <mergeCell ref="M63:M66"/>
+    <mergeCell ref="C205:C206"/>
     <mergeCell ref="B32:B35"/>
     <mergeCell ref="A207:A208"/>
     <mergeCell ref="A67:A70"/>
@@ -7941,13 +8173,16 @@
     <mergeCell ref="B46:B49"/>
     <mergeCell ref="E67:E70"/>
     <mergeCell ref="D150:D156"/>
+    <mergeCell ref="A215:A217"/>
     <mergeCell ref="B143:B149"/>
     <mergeCell ref="D183:D188"/>
     <mergeCell ref="A205:A206"/>
+    <mergeCell ref="M215:M217"/>
     <mergeCell ref="D125:D135"/>
     <mergeCell ref="A23:A31"/>
     <mergeCell ref="A143:A149"/>
     <mergeCell ref="C183:C188"/>
+    <mergeCell ref="B212:B214"/>
     <mergeCell ref="M46:M49"/>
     <mergeCell ref="M177:M179"/>
     <mergeCell ref="B10:B13"/>
@@ -7982,6 +8217,7 @@
     <mergeCell ref="B189:B194"/>
     <mergeCell ref="B71:B81"/>
     <mergeCell ref="M4:M9"/>
+    <mergeCell ref="D215:D217"/>
     <mergeCell ref="C43:C45"/>
     <mergeCell ref="A56:A62"/>
     <mergeCell ref="C56:C62"/>
@@ -7991,7 +8227,7 @@
     <mergeCell ref="A209:A211"/>
     <mergeCell ref="C209:C211"/>
     <mergeCell ref="B82:B92"/>
-    <mergeCell ref="C205:C206"/>
+    <mergeCell ref="E212:E214"/>
     <mergeCell ref="D143:D149"/>
     <mergeCell ref="C63:C66"/>
     <mergeCell ref="M67:M70"/>

</xml_diff>

<commit_message>
feat: PUSH LIST REV3 — texto maior, 2 zonas de foto por card, filtros e gráfico compacto
- Fonte aumentada: body 14px, nome-local 15px, meta 12px, tabela atividades 13px
- Mantém esquema de cores dark navy da REV2
- KPI "Ações Atrasadas" (atividades com previsão vencida e não concluídas)
- Gráfico de disciplinas compacto (34px/linha) embutido na seção de KPIs
- Barra de filtros restaurada: ÁREA · DISCIPLINA · STATUS · BUSCA com JavaScript
- Cada card com 2 zonas de foto lado a lado: ANTES/LEVANTAMENTO + PÓS/REALIZADO
- 38 cards · 214 atividades · Platô Central com 3 fotos

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168LAty28evK8EwJcgZFrtt
</commit_message>
<xml_diff>
--- a/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
+++ b/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Push List REV2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Push List REV3" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -556,17 +556,17 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -579,7 +579,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV2 — 03/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
+          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV3 — 03/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
         </is>
       </c>
     </row>
@@ -596,12 +596,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Local Nº</t>
+          <t>Local</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Nome do Local</t>
+          <t>Nome</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t># Ativ.</t>
+          <t>#Atv</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Atividade / Descrição</t>
+          <t>Atividade</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Avanço (%)</t>
+          <t>Avanço(%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: atualiza Excel REV3 com cabeçalhos e larguras de coluna iguais ao REV1
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168LAty28evK8EwJcgZFrtt
</commit_message>
<xml_diff>
--- a/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
+++ b/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
@@ -556,17 +556,17 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -596,12 +596,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Local Nº</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Nome</t>
+          <t>Nome do Local</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>#Atv</t>
+          <t># Ativ.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Atividade</t>
+          <t>Atividade / Descrição</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Avanço(%)</t>
+          <t>Avanço (%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Excel REV3 — tema claro (fundo branco/azul claro, texto escuro legível)
- Linha de dados: fundo branco (#FFFFFF) e azul clarinho (#EEF4FF) alternado
- Cabeçalho: azul médio (#1E4D99) com texto branco
- Título: azul navy (#1A3A6A) com texto branco
- Status Concluído: verde claro (#C8F0D8) / texto verde escuro
- Status Em andamento: âmbar claro (#FFF3CD) / texto escuro
- Avanço %: idem por faixa

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168LAty28evK8EwJcgZFrtt
</commit_message>
<xml_diff>
--- a/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
+++ b/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
@@ -28,32 +28,32 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0000BCD4"/>
+      <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="007BAFD4"/>
+      <color rgb="001A3A6A"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0000BCD4"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00C8D8F0"/>
+      <color rgb="001A2A40"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00B0BEC5"/>
+      <color rgb="005A7090"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -62,22 +62,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000A1628"/>
+        <fgColor rgb="001A3A6A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000D2540"/>
+        <fgColor rgb="00D6E4F7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000D1A30"/>
+        <fgColor rgb="001E4D99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00081020"/>
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF4FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,35 +96,35 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="0000BCD4"/>
+        <color rgb="001E4D99"/>
       </left>
       <right style="medium">
-        <color rgb="0000BCD4"/>
+        <color rgb="001E4D99"/>
       </right>
       <top style="medium">
-        <color rgb="0000BCD4"/>
+        <color rgb="001E4D99"/>
       </top>
       <bottom style="medium">
-        <color rgb="0000BCD4"/>
+        <color rgb="001E4D99"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </left>
       <right style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </right>
       <top style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </top>
       <bottom style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </left>
       <right/>
       <top/>
@@ -128,10 +133,10 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </left>
       <right style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </right>
       <top/>
       <bottom/>
@@ -139,14 +144,14 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </left>
       <right style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="001A3A60"/>
+        <color rgb="00BDD0E8"/>
       </bottom>
       <diagonal/>
     </border>
@@ -162,27 +167,14 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -193,8 +185,21 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -559,6 +564,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001565C0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -574,27 +580,27 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PUSH LIST — SERVIÇOS DAENG | ASU JUNDIAÍ (26001) | OTZ Engenharia × Messer Gases for Life</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV3 — 03/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>#Card</t>

</xml_diff>

<commit_message>
Push List REV3 — atualização 08/07/2026 (Excel 5 ATUALIZADO)
- TODAY = 08/07/2026 (dia 4/12 úteis)
- EXCEL_IN: 304d1831-DAENG_PUSH_LIST_ASU_JUNDIAI_5__ATUALIZADO_08.07.xlsx
- Excel já contém cards CFTV (C01–C12): removida chamada build_cftv_cards()
- build_cards() refatorado: detecta lnum "C..." e usa cftv_photos/ com landscape crop
- KPIs: 49 cards | 225 atv | 48 Concluídas | Avanço 21.3% | Previsto 33% | Defasagem 12.0 pp

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168LAty28evK8EwJcgZFrtt
</commit_message>
<xml_diff>
--- a/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
+++ b/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
@@ -623,7 +623,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV3 — 07/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
+          <t>Ref: CLM-216  |  Contratada: Andrade e Rocha (DAENG)  |  Gerenciadora: OTZ Engenharia — GPLAN  |  Levantamento: 02/07/2026  |  REV3 — 08/07/2026  |  Elaborado por: Ilson do Santos Azevedo / Supervisor de Planejamento</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,11 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>33.3%</t>
+        </is>
+      </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
           <t>33.3%</t>
@@ -927,15 +931,19 @@
       <c r="I10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="14" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
@@ -1072,10 +1080,14 @@
           <t>Concluída</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="9" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>44.4%</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -1131,9 +1143,9 @@
       <c r="I16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr"/>
@@ -1191,9 +1203,9 @@
       <c r="I18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
@@ -1362,10 +1374,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K23" s="11" t="inlineStr"/>
-      <c r="L23" s="15" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>22.2%</t>
         </is>
       </c>
     </row>
@@ -1391,9 +1407,9 @@
       <c r="I24" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr"/>
@@ -1571,9 +1587,9 @@
       <c r="I30" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J30" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr"/>
@@ -1652,7 +1668,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L32" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -1792,10 +1812,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr"/>
-      <c r="L36" s="14" t="inlineStr">
+      <c r="K36" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L36" s="9" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -1821,9 +1845,9 @@
       <c r="I37" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J37" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K37" s="11" t="inlineStr"/>
@@ -1902,10 +1926,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K39" s="11" t="inlineStr"/>
-      <c r="L39" s="15" t="inlineStr">
+      <c r="K39" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L39" s="9" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -1931,9 +1959,9 @@
       <c r="I40" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J40" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr"/>
@@ -2007,15 +2035,19 @@
       <c r="I42" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J42" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="14" t="inlineStr">
+      <c r="J42" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L42" s="8" t="inlineStr">
+        <is>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
@@ -2041,9 +2073,9 @@
       <c r="I43" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J43" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K43" s="11" t="inlineStr"/>
@@ -2071,9 +2103,9 @@
       <c r="I44" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J44" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J44" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr"/>
@@ -2152,7 +2184,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K46" s="4" t="inlineStr"/>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L46" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -2352,7 +2388,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K52" s="4" t="inlineStr"/>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L52" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -2582,7 +2622,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K59" s="11" t="inlineStr"/>
+      <c r="K59" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L59" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -2722,7 +2766,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K63" s="11" t="inlineStr"/>
+      <c r="K63" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L63" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -2862,7 +2910,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K67" s="11" t="inlineStr"/>
+      <c r="K67" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L67" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -3212,7 +3264,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K78" s="4" t="inlineStr"/>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L78" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -3562,7 +3618,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K89" s="11" t="inlineStr"/>
+      <c r="K89" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L89" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -3792,10 +3852,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K96" s="4" t="inlineStr"/>
-      <c r="L96" s="14" t="inlineStr">
+      <c r="K96" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L96" s="9" t="inlineStr">
+        <is>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
@@ -3941,9 +4005,9 @@
       <c r="I101" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J101" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J101" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K101" s="11" t="inlineStr"/>
@@ -3971,9 +4035,9 @@
       <c r="I102" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J102" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J102" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K102" s="4" t="inlineStr"/>
@@ -4142,10 +4206,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K107" s="11" t="inlineStr"/>
-      <c r="L107" s="15" t="inlineStr">
+      <c r="K107" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L107" s="9" t="inlineStr">
+        <is>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -4171,9 +4239,9 @@
       <c r="I108" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J108" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J108" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K108" s="4" t="inlineStr"/>
@@ -4261,9 +4329,9 @@
       <c r="I111" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J111" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J111" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K111" s="11" t="inlineStr"/>
@@ -4372,10 +4440,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K114" s="4" t="inlineStr"/>
-      <c r="L114" s="14" t="inlineStr">
+      <c r="K114" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L114" s="9" t="inlineStr">
+        <is>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -4431,9 +4503,9 @@
       <c r="I116" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J116" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J116" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K116" s="4" t="inlineStr"/>
@@ -4491,9 +4563,9 @@
       <c r="I118" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J118" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J118" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K118" s="4" t="inlineStr"/>
@@ -4602,10 +4674,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K121" s="11" t="inlineStr"/>
-      <c r="L121" s="15" t="inlineStr">
+      <c r="K121" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L121" s="9" t="inlineStr">
+        <is>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
@@ -4751,9 +4827,9 @@
       <c r="I126" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J126" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J126" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K126" s="4" t="inlineStr"/>
@@ -4841,9 +4917,9 @@
       <c r="I129" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J129" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J129" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K129" s="11" t="inlineStr"/>
@@ -4952,10 +5028,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K132" s="4" t="inlineStr"/>
-      <c r="L132" s="14" t="inlineStr">
+      <c r="K132" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L132" s="9" t="inlineStr">
+        <is>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -4981,9 +5061,9 @@
       <c r="I133" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J133" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J133" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K133" s="11" t="inlineStr"/>
@@ -5071,9 +5151,9 @@
       <c r="I136" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J136" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J136" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K136" s="4" t="inlineStr"/>
@@ -5182,10 +5262,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K139" s="11" t="inlineStr"/>
-      <c r="L139" s="15" t="inlineStr">
+      <c r="K139" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L139" s="9" t="inlineStr">
+        <is>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -5211,9 +5295,9 @@
       <c r="I140" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J140" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J140" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K140" s="4" t="inlineStr"/>
@@ -5301,9 +5385,9 @@
       <c r="I143" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J143" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J143" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K143" s="11" t="inlineStr"/>
@@ -5412,10 +5496,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K146" s="4" t="inlineStr"/>
-      <c r="L146" s="14" t="inlineStr">
+      <c r="K146" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L146" s="9" t="inlineStr">
+        <is>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -5441,9 +5529,9 @@
       <c r="I147" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J147" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J147" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K147" s="11" t="inlineStr"/>
@@ -5531,9 +5619,9 @@
       <c r="I150" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J150" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J150" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K150" s="4" t="inlineStr"/>
@@ -5642,10 +5730,14 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K153" s="11" t="inlineStr"/>
-      <c r="L153" s="15" t="inlineStr">
+      <c r="K153" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L153" s="9" t="inlineStr">
+        <is>
+          <t>18.2%</t>
         </is>
       </c>
     </row>
@@ -5791,9 +5883,9 @@
       <c r="I158" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J158" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J158" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K158" s="4" t="inlineStr"/>
@@ -5881,9 +5973,9 @@
       <c r="I161" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J161" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J161" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K161" s="11" t="inlineStr"/>
@@ -5992,7 +6084,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K164" s="4" t="inlineStr"/>
+      <c r="K164" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L164" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -6192,7 +6288,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K170" s="4" t="inlineStr"/>
+      <c r="K170" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L170" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -6302,7 +6402,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K173" s="11" t="inlineStr"/>
+      <c r="K173" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L173" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -6412,7 +6516,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K176" s="4" t="inlineStr"/>
+      <c r="K176" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L176" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -6517,15 +6625,19 @@
       <c r="I179" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J179" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K179" s="11" t="inlineStr"/>
-      <c r="L179" s="15" t="inlineStr">
+      <c r="J179" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K179" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L179" s="8" t="inlineStr">
+        <is>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -6551,9 +6663,9 @@
       <c r="I180" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J180" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J180" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K180" s="4" t="inlineStr"/>
@@ -6581,9 +6693,9 @@
       <c r="I181" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J181" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J181" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K181" s="11" t="inlineStr"/>
@@ -6641,9 +6753,9 @@
       <c r="I183" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J183" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J183" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K183" s="11" t="inlineStr"/>
@@ -6717,15 +6829,19 @@
       <c r="I185" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J185" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K185" s="11" t="inlineStr"/>
-      <c r="L185" s="15" t="inlineStr">
+      <c r="J185" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K185" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L185" s="8" t="inlineStr">
+        <is>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -6751,9 +6867,9 @@
       <c r="I186" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J186" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J186" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K186" s="4" t="inlineStr"/>
@@ -6781,9 +6897,9 @@
       <c r="I187" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J187" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J187" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K187" s="11" t="inlineStr"/>
@@ -6841,9 +6957,9 @@
       <c r="I189" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J189" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J189" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K189" s="11" t="inlineStr"/>
@@ -6917,15 +7033,19 @@
       <c r="I191" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J191" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K191" s="11" t="inlineStr"/>
-      <c r="L191" s="15" t="inlineStr">
+      <c r="J191" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K191" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L191" s="8" t="inlineStr">
+        <is>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -6951,9 +7071,9 @@
       <c r="I192" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J192" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J192" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K192" s="4" t="inlineStr"/>
@@ -6981,9 +7101,9 @@
       <c r="I193" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J193" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J193" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K193" s="11" t="inlineStr"/>
@@ -7041,9 +7161,9 @@
       <c r="I195" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J195" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="J195" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
         </is>
       </c>
       <c r="K195" s="11" t="inlineStr"/>
@@ -7122,7 +7242,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K197" s="11" t="inlineStr"/>
+      <c r="K197" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L197" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -7202,7 +7326,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K199" s="11" t="inlineStr"/>
+      <c r="K199" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L199" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -7282,7 +7410,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K201" s="11" t="inlineStr"/>
+      <c r="K201" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L201" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -7362,7 +7494,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K203" s="11" t="inlineStr"/>
+      <c r="K203" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L203" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -7437,15 +7573,19 @@
       <c r="I205" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J205" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K205" s="11" t="inlineStr"/>
-      <c r="L205" s="15" t="inlineStr">
+      <c r="J205" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K205" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L205" s="9" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -7552,7 +7692,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K208" s="4" t="inlineStr"/>
+      <c r="K208" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L208" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -7657,15 +7801,19 @@
       <c r="I211" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J211" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K211" s="11" t="inlineStr"/>
-      <c r="L211" s="15" t="inlineStr">
+      <c r="J211" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K211" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L211" s="9" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7920,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K214" s="4" t="inlineStr"/>
+      <c r="K214" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L214" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -7817,15 +7969,19 @@
       <c r="I215" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="J215" s="15" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K215" s="11" t="inlineStr"/>
-      <c r="L215" s="15" t="inlineStr">
+      <c r="J215" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K215" s="11" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L215" s="8" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -7867,15 +8023,19 @@
       <c r="I216" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J216" s="14" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="K216" s="4" t="inlineStr"/>
-      <c r="L216" s="14" t="inlineStr">
+      <c r="J216" s="8" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="K216" s="4" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L216" s="9" t="inlineStr">
+        <is>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -7952,7 +8112,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K218" s="4" t="inlineStr"/>
+      <c r="K218" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L218" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8002,7 +8166,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K219" s="11" t="inlineStr"/>
+      <c r="K219" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L219" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8052,7 +8220,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K220" s="4" t="inlineStr"/>
+      <c r="K220" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L220" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8102,7 +8274,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K221" s="11" t="inlineStr"/>
+      <c r="K221" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L221" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8152,7 +8328,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K222" s="4" t="inlineStr"/>
+      <c r="K222" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L222" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8202,7 +8382,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K223" s="11" t="inlineStr"/>
+      <c r="K223" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L223" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8312,7 +8496,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K226" s="4" t="inlineStr"/>
+      <c r="K226" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L226" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8362,7 +8550,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K227" s="11" t="inlineStr"/>
+      <c r="K227" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L227" s="15" t="inlineStr">
         <is>
           <t>0.0%</t>
@@ -8414,7 +8606,11 @@
           <t>Pendente</t>
         </is>
       </c>
-      <c r="K228" s="4" t="inlineStr"/>
+      <c r="K228" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
       <c r="L228" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>

</xml_diff>

<commit_message>
Push List REV3 — formalização e-mail: 6 melhorias aplicadas
1. Curva-S: subtítulo "Entrega de Documentação (Data Book)" em vermelho Messer
2. Excel: linha entregável "Data Book" (peso 0, sem impacto no avanço físico)
3. KPI novo: Data de Tendência (pendentes ÷ velocidade → data projetada, cal. seg-sáb)
4. Coluna Conclusão: Concluída = 100% / Pendente = data ou —
5. Reclassificação: "Macrodrenagem / 5S" → "Macrodrenagem" em HTML + Excel
6. PDF: versão impressa tema claro Messer (#1A3680 + #CC2020 + fundo branco)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0168LAty28evK8EwJcgZFrtt
</commit_message>
<xml_diff>
--- a/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
+++ b/projetos/OTZ_ASU_JUNDIAI/push_list/DAENG_PUSH_LIST_ASU_JUNDIAI.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,8 +64,24 @@
       <color rgb="005A7090"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A3680"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007B4F00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A3680"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +121,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF4FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8EAF8"/>
       </patternFill>
     </fill>
   </fills>
@@ -181,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -229,6 +250,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L228"/>
+  <dimension ref="A1:L229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1796,7 +1832,7 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -1834,7 +1870,7 @@
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H37" s="13" t="inlineStr">
@@ -1910,7 +1946,7 @@
       </c>
       <c r="G39" s="12" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H39" s="13" t="inlineStr">
@@ -1948,7 +1984,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
@@ -3172,7 +3208,7 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
@@ -3526,7 +3562,7 @@
       </c>
       <c r="G87" s="12" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H87" s="13" t="inlineStr">
@@ -3760,7 +3796,7 @@
       </c>
       <c r="G94" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
@@ -4114,7 +4150,7 @@
       </c>
       <c r="G105" s="12" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H105" s="13" t="inlineStr">
@@ -4348,7 +4384,7 @@
       </c>
       <c r="G112" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H112" s="7" t="inlineStr">
@@ -4582,7 +4618,7 @@
       </c>
       <c r="G119" s="12" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H119" s="13" t="inlineStr">
@@ -4936,7 +4972,7 @@
       </c>
       <c r="G130" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H130" s="7" t="inlineStr">
@@ -5170,7 +5206,7 @@
       </c>
       <c r="G137" s="12" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H137" s="13" t="inlineStr">
@@ -5404,7 +5440,7 @@
       </c>
       <c r="G144" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H144" s="7" t="inlineStr">
@@ -5638,7 +5674,7 @@
       </c>
       <c r="G151" s="12" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H151" s="13" t="inlineStr">
@@ -5992,7 +6028,7 @@
       </c>
       <c r="G162" s="6" t="inlineStr">
         <is>
-          <t>Macrodrenagem / 5S</t>
+          <t>Macrodrenagem</t>
         </is>
       </c>
       <c r="H162" s="7" t="inlineStr">
@@ -8614,6 +8650,66 @@
       <c r="L228" s="14" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="16" customHeight="1">
+      <c r="A229" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B229" s="19" t="inlineStr">
+        <is>
+          <t>Documentação</t>
+        </is>
+      </c>
+      <c r="C229" s="18" t="inlineStr">
+        <is>
+          <t>DOC</t>
+        </is>
+      </c>
+      <c r="D229" s="19" t="inlineStr">
+        <is>
+          <t>Entrega de Documentação (Data Book)</t>
+        </is>
+      </c>
+      <c r="E229" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F229" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G229" s="19" t="inlineStr">
+        <is>
+          <t>Contrato</t>
+        </is>
+      </c>
+      <c r="H229" s="20" t="inlineStr">
+        <is>
+          <t>Entrega do Data Book completo da obra</t>
+        </is>
+      </c>
+      <c r="I229" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J229" s="19" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="K229" s="18" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="L229" s="22" t="inlineStr">
+        <is>
+          <t>Entregável</t>
         </is>
       </c>
     </row>

</xml_diff>